<commit_message>
update metric, visualisasi model, visualisasi peta
</commit_message>
<xml_diff>
--- a/outputs/tables/ranking_top_bottom_2024.xlsx
+++ b/outputs/tables/ranking_top_bottom_2024.xlsx
@@ -15,6 +15,8 @@
     <sheet name="rasio_klinik_top" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="rasio_rsu_total_bottom" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="rasio_rsu_total_top" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="skor_layanan_bottom" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="skor_layanan_top" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -532,6 +534,112 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kab_kota</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>skor_layanan</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>kelas_layanan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>KOTA BANJAR</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1.749353437465112</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>KOTA CIREBON</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.138262906022369</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>KOTA SUKABUMI</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1.028243086502464</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>KOTA TASIKMALAYA</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.8367514557921856</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>KOTA BEKASI</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.6859181155107771</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1272,4 +1380,110 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kab_kota</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>skor_layanan</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>kelas_layanan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>KABUPATEN BANDUNG</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>-0.9102433986124744</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Rendah</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>KABUPATEN CIANJUR</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>-0.8430220850903997</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Rendah</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>KABUPATEN BANDUNG BARAT</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>-0.8229720773030615</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Rendah</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>KABUPATEN BOGOR</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>-0.7716932757697534</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Rendah</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>KABUPATEN TASIKMALAYA</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-0.6695548467784391</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Rendah</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>